<commit_message>
feat(account): add independent usernames and avatars
</commit_message>
<xml_diff>
--- a/PM/feature_progress.xlsx
+++ b/PM/feature_progress.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nine Dimensions" sheetId="1" r:id="R4ee3626ca8654f58"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="2" r:id="R39552afcd96c4118"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active Batch" sheetId="3" r:id="R964c07b94c2849c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Role Capacity" sheetId="4" r:id="R0bb01499ebee420a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Update Rules" sheetId="5" r:id="Rb23d57075fdc4b2b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nine Dimensions" sheetId="1" r:id="R4c42214f50fb4e06"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="2" r:id="Ra917492d25de45c7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active Batch" sheetId="3" r:id="R3913ec37d764425b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Role Capacity" sheetId="4" r:id="R7f249c308d8a4d5f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Update Rules" sheetId="5" r:id="R47976c76984c4371"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -103,7 +103,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="31">
+  <x:cellXfs count="33">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -163,6 +163,12 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -490,11 +496,11 @@
       </x:c>
       <x:c r="C6" s="12" t="n">
         <x:f>COUNTIF($H$18:$H$117,1)</x:f>
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="D6" s="12" t="n">
         <x:f>COUNT($H$18:$H$117)</x:f>
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="E6" s="12" t="str">
         <x:v>File behavior changes into a functional source</x:v>
@@ -526,15 +532,15 @@
       </x:c>
       <x:c r="B8" s="13" t="n">
         <x:f>IFERROR(AVERAGE($J$18:$J$117),0)</x:f>
-        <x:v>0.17</x:v>
+        <x:v>0.30833333333333335</x:v>
       </x:c>
       <x:c r="C8" s="12" t="n">
         <x:f>COUNTIF($J$18:$J$117,1)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D8" s="12" t="n">
         <x:f>COUNT($J$18:$J$117)</x:f>
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="E8" s="12" t="str">
         <x:v>Implement the real behavior path</x:v>
@@ -566,15 +572,15 @@
       </x:c>
       <x:c r="B10" s="13" t="n">
         <x:f>IFERROR(AVERAGE($L$18:$L$117),0)</x:f>
-        <x:v>0.2875</x:v>
+        <x:v>0.43</x:v>
       </x:c>
       <x:c r="C10" s="12" t="n">
         <x:f>COUNTIF($L$18:$L$117,1)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D10" s="12" t="n">
         <x:f>COUNT($L$18:$L$117)</x:f>
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="E10" s="12" t="str">
         <x:v>Define required interaction and feedback</x:v>
@@ -586,7 +592,7 @@
       </x:c>
       <x:c r="B11" s="13" t="n">
         <x:f>IFERROR(AVERAGE($M$18:$M$117),0)</x:f>
-        <x:v>0.44999999999999996</x:v>
+        <x:v>0.51</x:v>
       </x:c>
       <x:c r="C11" s="12" t="n">
         <x:f>COUNTIF($M$18:$M$117,1)</x:f>
@@ -594,7 +600,7 @@
       </x:c>
       <x:c r="D11" s="12" t="n">
         <x:f>COUNT($M$18:$M$117)</x:f>
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="E11" s="12" t="str">
         <x:v>Produce final-quality visual assets</x:v>
@@ -626,7 +632,7 @@
       </x:c>
       <x:c r="B13" s="13" t="n">
         <x:f>IFERROR(AVERAGE($O$18:$O$117),0)</x:f>
-        <x:v>0.025</x:v>
+        <x:v>0.16999999999999998</x:v>
       </x:c>
       <x:c r="C13" s="12" t="n">
         <x:f>COUNTIF($O$18:$O$117,1)</x:f>
@@ -634,7 +640,7 @@
       </x:c>
       <x:c r="D13" s="12" t="n">
         <x:f>COUNT($O$18:$O$117)</x:f>
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="E13" s="12" t="str">
         <x:v>Bind approved images to runtime behavior</x:v>
@@ -646,15 +652,15 @@
       </x:c>
       <x:c r="B14" s="13" t="n">
         <x:f>IFERROR(AVERAGE($P$18:$P$117),0)</x:f>
-        <x:v>0.175</x:v>
+        <x:v>0.33999999999999997</x:v>
       </x:c>
       <x:c r="C14" s="12" t="n">
         <x:f>COUNTIF($P$18:$P$117,1)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D14" s="12" t="n">
         <x:f>COUNT($P$18:$P$117)</x:f>
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="E14" s="12" t="str">
         <x:v>Complete functional UI behavior</x:v>
@@ -665,7 +671,8 @@
         <x:v>Feature total</x:v>
       </x:c>
       <x:c r="B15" s="12" t="n">
-        <x:v>5</x:v>
+        <x:f>COUNTA($A$18:$A$117)</x:f>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C15" s="12" t="n">
         <x:f>COUNTIF($Q$18:$Q$117,1)</x:f>
@@ -673,7 +680,7 @@
       </x:c>
       <x:c r="D15" s="13" t="n">
         <x:f>IFERROR(AVERAGE($Q$18:$Q$117),0)</x:f>
-        <x:v>0.4066666666666666</x:v>
+        <x:v>0.49166666666666664</x:v>
       </x:c>
       <x:c r="E15" s="12" t="str">
         <x:v>Overall averages applicable dimensions per feature</x:v>
@@ -1072,6 +1079,72 @@
       </x:c>
       <x:c r="U22" s="21" t="str">
         <x:v>Final assets incomplete</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="118" customHeight="1">
+      <x:c r="A23" s="32" t="str">
+        <x:v>F-ZC-AUTH-001</x:v>
+      </x:c>
+      <x:c r="B23" s="32" t="str">
+        <x:v>Player account identity, username, avatar and credential copy</x:v>
+      </x:c>
+      <x:c r="C23" s="32" t="str">
+        <x:v>General design DOCX + runtime code + review board</x:v>
+      </x:c>
+      <x:c r="D23" s="32" t="str">
+        <x:v>docs/PLAYER_ACCOUNT_IDENTITY_AVATAR_DESIGN_v2.0.docx</x:v>
+      </x:c>
+      <x:c r="E23" s="32" t="str">
+        <x:v>Not needed</x:v>
+      </x:c>
+      <x:c r="F23" s="32" t="str">
+        <x:v>Keep account ID stable; username is an independent display name; retain direct login and three credential copy actions</x:v>
+      </x:c>
+      <x:c r="G23" s="32" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="H23" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I23" s="32" t="str">
+        <x:v>Not needed</x:v>
+      </x:c>
+      <x:c r="J23" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K23" s="32" t="str">
+        <x:v>Not needed</x:v>
+      </x:c>
+      <x:c r="L23" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M23" s="32" t="n">
+        <x:v>0.75</x:v>
+      </x:c>
+      <x:c r="N23" s="32" t="str">
+        <x:v>Not needed</x:v>
+      </x:c>
+      <x:c r="O23" s="32" t="n">
+        <x:v>0.75</x:v>
+      </x:c>
+      <x:c r="P23" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Q23" s="32" t="n">
+        <x:f>AVERAGE(H23:P23)</x:f>
+        <x:v>0.9166666666666666</x:v>
+      </x:c>
+      <x:c r="R23" s="32" t="str">
+        <x:v>Local implementation complete</x:v>
+      </x:c>
+      <x:c r="S23" s="32" t="str">
+        <x:v>Design / Engineering / Art</x:v>
+      </x:c>
+      <x:c r="T23" s="32" t="str">
+        <x:v>Producer approval for the human avatar board; production auth hardening</x:v>
+      </x:c>
+      <x:c r="U23" s="32" t="str">
+        <x:v>FigJam unavailable; human portraits NOT_RUNTIME; KDF/TLS/rate-limit/Aliyun authorization pending</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1162,7 +1235,8 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="27" t="n">
-        <x:v>3</x:v>
+        <x:f>COUNTA('Nine Dimensions'!$A$18:$A$117)</x:f>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="B5" s="27" t="n">
         <x:v>0</x:v>

</xml_diff>